<commit_message>
Fixed BWP and Commands
</commit_message>
<xml_diff>
--- a/app/nsa_sa/DB.xlsx
+++ b/app/nsa_sa/DB.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aj_mac/Documents/Atel/server/code/app/nsa_sa/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aj_mac/Documents/Atel/server_new/app/nsa_sa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCFC4D4-098C-974E-8EB9-77AA6D2B9B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527E5214-0A7E-CA4A-92DF-9B62147E95F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16080" firstSheet="1" activeTab="5" xr2:uid="{0D659C63-0EA7-475F-99B7-E7E648DB9099}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="MOC" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">MOC!$A$1:$G$286</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">MOC!$A$1:$G$318</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2923" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2931" uniqueCount="538">
   <si>
     <t>5qi1</t>
   </si>
@@ -1650,6 +1650,12 @@
   </si>
   <si>
     <t>{"mappingInfoSIB24": "MAPPED_SI_1"}</t>
+  </si>
+  <si>
+    <t>zzzTemporary1</t>
+  </si>
+  <si>
+    <t>ENodeBFunction=1,UePolicyOptimization=1</t>
   </si>
 </sst>
 </file>
@@ -1692,7 +1698,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1729,6 +1735,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1757,7 +1769,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1771,6 +1783,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5813,7 +5826,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04129BFA-1C57-4A9F-9E8B-6ECAA0BFBBBF}">
-  <dimension ref="A1:H317"/>
+  <dimension ref="A1:H318"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" style="8" bestFit="1" customWidth="1"/>
@@ -6009,172 +6022,174 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="A8" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>506</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>494</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>355</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="3"/>
+      <c r="G8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="3"/>
+      <c r="A9" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="3"/>
+      <c r="A10" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="11"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="3"/>
+      <c r="A11" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="3"/>
+      <c r="A12" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="11"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="3"/>
+      <c r="A13" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="3"/>
+      <c r="A14" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
@@ -6187,7 +6202,7 @@
         <v>506</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>355</v>
@@ -6211,7 +6226,7 @@
         <v>506</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>355</v>
@@ -6235,7 +6250,7 @@
         <v>506</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>355</v>
@@ -6259,7 +6274,7 @@
         <v>506</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>355</v>
@@ -6283,7 +6298,7 @@
         <v>506</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>355</v>
@@ -6307,7 +6322,7 @@
         <v>506</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>355</v>
@@ -6331,7 +6346,7 @@
         <v>506</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>355</v>
@@ -6355,7 +6370,7 @@
         <v>506</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>355</v>
@@ -6379,7 +6394,7 @@
         <v>506</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>355</v>
@@ -6403,7 +6418,7 @@
         <v>506</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>355</v>
@@ -6427,7 +6442,7 @@
         <v>506</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>355</v>
@@ -6451,7 +6466,7 @@
         <v>506</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>355</v>
@@ -6475,7 +6490,7 @@
         <v>506</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>355</v>
@@ -6499,7 +6514,7 @@
         <v>506</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>355</v>
@@ -6523,7 +6538,7 @@
         <v>506</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>355</v>
@@ -6547,7 +6562,7 @@
         <v>506</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>494</v>
+        <v>411</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>355</v>
@@ -6571,7 +6586,7 @@
         <v>506</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>495</v>
+        <v>412</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>355</v>
@@ -6595,7 +6610,7 @@
         <v>506</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>496</v>
+        <v>413</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>355</v>
@@ -6619,7 +6634,7 @@
         <v>506</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>497</v>
+        <v>414</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>355</v>
@@ -6643,7 +6658,7 @@
         <v>506</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>498</v>
+        <v>415</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>355</v>
@@ -6667,13 +6682,13 @@
         <v>506</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>164</v>
+        <v>416</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>165</v>
+        <v>355</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>168</v>
+        <v>393</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>17</v>
@@ -6691,13 +6706,13 @@
         <v>506</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>164</v>
+        <v>417</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>166</v>
+        <v>355</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>17</v>
+        <v>393</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>17</v>
@@ -6715,13 +6730,13 @@
         <v>506</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>167</v>
+        <v>495</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>165</v>
+        <v>355</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>168</v>
+        <v>393</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>17</v>
@@ -6739,13 +6754,13 @@
         <v>506</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>167</v>
+        <v>496</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>166</v>
+        <v>355</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>17</v>
+        <v>393</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>17</v>
@@ -6763,13 +6778,13 @@
         <v>506</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>313</v>
+        <v>497</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>314</v>
+        <v>355</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>17</v>
+        <v>393</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>17</v>
@@ -6787,13 +6802,13 @@
         <v>506</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>315</v>
+        <v>498</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>316</v>
+        <v>355</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>379</v>
+        <v>393</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>17</v>
@@ -6811,13 +6826,13 @@
         <v>506</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>315</v>
+        <v>164</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>317</v>
+        <v>165</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>16</v>
+        <v>168</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>17</v>
@@ -6835,13 +6850,13 @@
         <v>506</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>315</v>
+        <v>164</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>318</v>
+        <v>166</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>17</v>
@@ -6859,13 +6874,13 @@
         <v>506</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>315</v>
+        <v>167</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>319</v>
+        <v>165</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>17</v>
@@ -6883,13 +6898,13 @@
         <v>506</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>315</v>
+        <v>167</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>320</v>
+        <v>166</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>17</v>
@@ -6907,13 +6922,13 @@
         <v>506</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>338</v>
+        <v>313</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F45" s="3">
-        <v>34</v>
+        <v>314</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>17</v>
@@ -6931,13 +6946,13 @@
         <v>506</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>339</v>
+        <v>315</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F46" s="3">
-        <v>34</v>
+        <v>316</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>379</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>17</v>
@@ -6955,13 +6970,13 @@
         <v>506</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F47" s="3">
-        <v>12</v>
+        <v>317</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>17</v>
@@ -6979,13 +6994,13 @@
         <v>506</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>341</v>
+        <v>315</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F48" s="3">
-        <v>12</v>
+        <v>318</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>17</v>
@@ -7003,13 +7018,13 @@
         <v>506</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F49" s="3">
-        <v>46</v>
+        <v>319</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>193</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>17</v>
@@ -7027,13 +7042,13 @@
         <v>506</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>343</v>
+        <v>315</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F50" s="3">
-        <v>32</v>
+        <v>320</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>17</v>
@@ -7051,13 +7066,13 @@
         <v>506</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>93</v>
       </c>
       <c r="F51" s="3">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>17</v>
@@ -7075,13 +7090,13 @@
         <v>506</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>93</v>
       </c>
       <c r="F52" s="3">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>17</v>
@@ -7099,13 +7114,13 @@
         <v>506</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>93</v>
       </c>
       <c r="F53" s="3">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>17</v>
@@ -7123,13 +7138,13 @@
         <v>506</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>139</v>
+        <v>341</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>158</v>
+        <v>93</v>
+      </c>
+      <c r="F54" s="3">
+        <v>12</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>17</v>
@@ -7147,13 +7162,13 @@
         <v>506</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>139</v>
+        <v>342</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>158</v>
+        <v>93</v>
+      </c>
+      <c r="F55" s="3">
+        <v>46</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>17</v>
@@ -7171,13 +7186,13 @@
         <v>506</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>139</v>
+        <v>343</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>123</v>
+        <v>93</v>
+      </c>
+      <c r="F56" s="3">
+        <v>32</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>17</v>
@@ -7195,13 +7210,13 @@
         <v>506</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>139</v>
+        <v>344</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>58</v>
+        <v>93</v>
+      </c>
+      <c r="F57" s="3">
+        <v>40</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>17</v>
@@ -7219,13 +7234,13 @@
         <v>506</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>139</v>
+        <v>345</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>17</v>
+        <v>93</v>
+      </c>
+      <c r="F58" s="3">
+        <v>30</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>17</v>
@@ -7243,13 +7258,13 @@
         <v>506</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>139</v>
+        <v>346</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>380</v>
+        <v>93</v>
+      </c>
+      <c r="F59" s="3">
+        <v>26</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>17</v>
@@ -7267,13 +7282,13 @@
         <v>506</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>17</v>
@@ -7291,13 +7306,13 @@
         <v>506</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>17</v>
@@ -7315,10 +7330,10 @@
         <v>506</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>123</v>
@@ -7339,13 +7354,13 @@
         <v>506</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>17</v>
@@ -7363,10 +7378,10 @@
         <v>506</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>17</v>
@@ -7387,13 +7402,13 @@
         <v>506</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>17</v>
@@ -7411,13 +7426,13 @@
         <v>506</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>17</v>
+        <v>162</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>17</v>
@@ -7435,13 +7450,13 @@
         <v>506</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>17</v>
+        <v>163</v>
       </c>
       <c r="G67" s="3" t="s">
         <v>17</v>
@@ -7459,13 +7474,13 @@
         <v>506</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>17</v>
+        <v>123</v>
       </c>
       <c r="G68" s="3" t="s">
         <v>17</v>
@@ -7483,13 +7498,13 @@
         <v>506</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="G69" s="3" t="s">
         <v>17</v>
@@ -7507,13 +7522,13 @@
         <v>506</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>232</v>
+        <v>153</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>85</v>
+        <v>154</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="G70" s="3" t="s">
         <v>17</v>
@@ -7531,13 +7546,13 @@
         <v>506</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>232</v>
+        <v>153</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>297</v>
+        <v>155</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>17</v>
+        <v>381</v>
       </c>
       <c r="G71" s="3" t="s">
         <v>17</v>
@@ -7555,13 +7570,13 @@
         <v>506</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>233</v>
+        <v>153</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>234</v>
+        <v>156</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>123</v>
+        <v>17</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>17</v>
@@ -7579,13 +7594,13 @@
         <v>506</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>476</v>
+        <v>153</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>234</v>
+        <v>157</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>477</v>
+        <v>17</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>17</v>
@@ -7603,13 +7618,13 @@
         <v>506</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>476</v>
+        <v>149</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>478</v>
+        <v>150</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>123</v>
+        <v>17</v>
       </c>
       <c r="G74" s="3" t="s">
         <v>17</v>
@@ -7627,13 +7642,13 @@
         <v>506</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>476</v>
+        <v>151</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>479</v>
+        <v>152</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>123</v>
+        <v>17</v>
       </c>
       <c r="G75" s="3" t="s">
         <v>17</v>
@@ -7651,13 +7666,13 @@
         <v>506</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>476</v>
+        <v>232</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>269</v>
+        <v>85</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>255</v>
+        <v>72</v>
       </c>
       <c r="G76" s="3" t="s">
         <v>17</v>
@@ -7675,10 +7690,10 @@
         <v>506</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>248</v>
+        <v>232</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>247</v>
+        <v>297</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>17</v>
@@ -7699,13 +7714,13 @@
         <v>506</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>17</v>
+        <v>123</v>
       </c>
       <c r="G78" s="3" t="s">
         <v>17</v>
@@ -7723,13 +7738,13 @@
         <v>506</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>235</v>
+        <v>476</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>382</v>
+        <v>477</v>
       </c>
       <c r="G79" s="3" t="s">
         <v>17</v>
@@ -7747,13 +7762,13 @@
         <v>506</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>235</v>
+        <v>476</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>237</v>
+        <v>478</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>238</v>
+        <v>123</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>17</v>
@@ -7771,13 +7786,13 @@
         <v>506</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>235</v>
+        <v>476</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>239</v>
+        <v>479</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>383</v>
+        <v>123</v>
       </c>
       <c r="G81" s="3" t="s">
         <v>17</v>
@@ -7795,13 +7810,13 @@
         <v>506</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>235</v>
+        <v>476</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>383</v>
+        <v>255</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>17</v>
@@ -7819,13 +7834,13 @@
         <v>506</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G83" s="3" t="s">
         <v>17</v>
@@ -7843,13 +7858,13 @@
         <v>506</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>384</v>
+        <v>17</v>
       </c>
       <c r="G84" s="3" t="s">
         <v>17</v>
@@ -7870,10 +7885,10 @@
         <v>235</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>244</v>
+        <v>382</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>17</v>
@@ -7894,10 +7909,10 @@
         <v>235</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>17</v>
@@ -7915,13 +7930,13 @@
         <v>506</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>119</v>
+        <v>235</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>120</v>
+        <v>239</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>17</v>
+        <v>383</v>
       </c>
       <c r="G87" s="3" t="s">
         <v>17</v>
@@ -7939,13 +7954,13 @@
         <v>506</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>119</v>
+        <v>235</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>121</v>
+        <v>240</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>56</v>
+        <v>383</v>
       </c>
       <c r="G88" s="3" t="s">
         <v>17</v>
@@ -7963,13 +7978,13 @@
         <v>506</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>119</v>
+        <v>235</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>122</v>
+        <v>241</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>123</v>
+        <v>18</v>
       </c>
       <c r="G89" s="3" t="s">
         <v>17</v>
@@ -7987,13 +8002,13 @@
         <v>506</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>124</v>
+        <v>235</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>125</v>
+        <v>242</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>72</v>
+        <v>384</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>17</v>
@@ -8011,13 +8026,13 @@
         <v>506</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>126</v>
+        <v>235</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>127</v>
+        <v>243</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>16</v>
+        <v>244</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>17</v>
@@ -8035,13 +8050,13 @@
         <v>506</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>126</v>
+        <v>235</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>128</v>
+        <v>245</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>395</v>
+        <v>246</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>17</v>
@@ -8059,13 +8074,13 @@
         <v>506</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>253</v>
+        <v>119</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>254</v>
+        <v>120</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>255</v>
+        <v>17</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>17</v>
@@ -8083,13 +8098,13 @@
         <v>506</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>275</v>
+        <v>119</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>276</v>
+        <v>121</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>255</v>
+        <v>56</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>17</v>
@@ -8107,13 +8122,13 @@
         <v>506</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>275</v>
+        <v>119</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>277</v>
+        <v>122</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>255</v>
+        <v>123</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>17</v>
@@ -8131,12 +8146,14 @@
         <v>506</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>252</v>
+        <v>124</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="F96" s="3"/>
+        <v>125</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="G96" s="3" t="s">
         <v>17</v>
       </c>
@@ -8153,13 +8170,13 @@
         <v>506</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>295</v>
+        <v>126</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>280</v>
+        <v>127</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>384</v>
+        <v>16</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>17</v>
@@ -8177,13 +8194,13 @@
         <v>506</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>295</v>
+        <v>126</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>281</v>
+        <v>128</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>17</v>
+        <v>395</v>
       </c>
       <c r="G98" s="3" t="s">
         <v>17</v>
@@ -8201,13 +8218,13 @@
         <v>506</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>295</v>
+        <v>253</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>73</v>
+        <v>255</v>
       </c>
       <c r="G99" s="3" t="s">
         <v>17</v>
@@ -8225,13 +8242,13 @@
         <v>506</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>285</v>
+        <v>255</v>
       </c>
       <c r="G100" s="3" t="s">
         <v>17</v>
@@ -8249,13 +8266,13 @@
         <v>506</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>421</v>
+        <v>255</v>
       </c>
       <c r="G101" s="3" t="s">
         <v>17</v>
@@ -8273,14 +8290,12 @@
         <v>506</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>295</v>
+        <v>252</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="F102" s="3" t="s">
-        <v>290</v>
-      </c>
+        <v>279</v>
+      </c>
+      <c r="F102" s="3"/>
       <c r="G102" s="3" t="s">
         <v>17</v>
       </c>
@@ -8300,10 +8315,10 @@
         <v>295</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>291</v>
+        <v>384</v>
       </c>
       <c r="G103" s="3" t="s">
         <v>17</v>
@@ -8321,13 +8336,13 @@
         <v>506</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>384</v>
+        <v>17</v>
       </c>
       <c r="G104" s="3" t="s">
         <v>17</v>
@@ -8345,13 +8360,13 @@
         <v>506</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="G105" s="3" t="s">
         <v>17</v>
@@ -8369,13 +8384,13 @@
         <v>506</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>73</v>
+        <v>285</v>
       </c>
       <c r="G106" s="3" t="s">
         <v>17</v>
@@ -8393,13 +8408,13 @@
         <v>506</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>283</v>
+        <v>421</v>
       </c>
       <c r="G107" s="3" t="s">
         <v>17</v>
@@ -8417,13 +8432,13 @@
         <v>506</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>255</v>
+        <v>290</v>
       </c>
       <c r="G108" s="3" t="s">
         <v>17</v>
@@ -8441,13 +8456,13 @@
         <v>506</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="G109" s="3" t="s">
         <v>17</v>
@@ -8468,10 +8483,10 @@
         <v>296</v>
       </c>
       <c r="E110" s="3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>292</v>
+        <v>384</v>
       </c>
       <c r="G110" s="3" t="s">
         <v>17</v>
@@ -8492,10 +8507,10 @@
         <v>296</v>
       </c>
       <c r="E111" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>293</v>
+        <v>18</v>
       </c>
       <c r="G111" s="3" t="s">
         <v>17</v>
@@ -8516,10 +8531,10 @@
         <v>296</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>294</v>
+        <v>73</v>
       </c>
       <c r="G112" s="3" t="s">
         <v>17</v>
@@ -8537,13 +8552,13 @@
         <v>506</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>322</v>
+        <v>268</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>16</v>
+        <v>283</v>
       </c>
       <c r="G113" s="3" t="s">
         <v>17</v>
@@ -8561,13 +8576,13 @@
         <v>506</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>323</v>
+        <v>269</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>158</v>
+        <v>255</v>
       </c>
       <c r="G114" s="3" t="s">
         <v>17</v>
@@ -8585,13 +8600,13 @@
         <v>506</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>324</v>
+        <v>284</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>17</v>
+        <v>286</v>
       </c>
       <c r="G115" s="3" t="s">
         <v>17</v>
@@ -8609,13 +8624,13 @@
         <v>506</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>325</v>
+        <v>292</v>
       </c>
       <c r="G116" s="3" t="s">
         <v>17</v>
@@ -8633,13 +8648,13 @@
         <v>506</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>325</v>
+        <v>293</v>
       </c>
       <c r="G117" s="3" t="s">
         <v>17</v>
@@ -8657,13 +8672,13 @@
         <v>506</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>326</v>
+        <v>296</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>322</v>
+        <v>289</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>16</v>
+        <v>294</v>
       </c>
       <c r="G118" s="3" t="s">
         <v>17</v>
@@ -8681,13 +8696,13 @@
         <v>506</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>158</v>
+        <v>16</v>
       </c>
       <c r="G119" s="3" t="s">
         <v>17</v>
@@ -8705,13 +8720,13 @@
         <v>506</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="G120" s="3" t="s">
         <v>17</v>
@@ -8729,13 +8744,13 @@
         <v>506</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E121" s="3" t="s">
-        <v>268</v>
+        <v>324</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>327</v>
+        <v>17</v>
       </c>
       <c r="G121" s="3" t="s">
         <v>17</v>
@@ -8753,13 +8768,13 @@
         <v>506</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="G122" s="3" t="s">
         <v>17</v>
@@ -8777,13 +8792,13 @@
         <v>506</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>322</v>
+        <v>269</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>16</v>
+        <v>325</v>
       </c>
       <c r="G123" s="3" t="s">
         <v>17</v>
@@ -8801,13 +8816,13 @@
         <v>506</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>158</v>
+        <v>16</v>
       </c>
       <c r="G124" s="3" t="s">
         <v>17</v>
@@ -8825,13 +8840,13 @@
         <v>506</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>17</v>
+        <v>158</v>
       </c>
       <c r="G125" s="3" t="s">
         <v>17</v>
@@ -8849,13 +8864,13 @@
         <v>506</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>268</v>
+        <v>324</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>329</v>
+        <v>18</v>
       </c>
       <c r="G126" s="3" t="s">
         <v>17</v>
@@ -8873,13 +8888,13 @@
         <v>506</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="G127" s="3" t="s">
         <v>17</v>
@@ -8897,13 +8912,13 @@
         <v>506</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>454</v>
+        <v>326</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>455</v>
+        <v>269</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>456</v>
+        <v>327</v>
       </c>
       <c r="G128" s="3" t="s">
         <v>17</v>
@@ -8921,13 +8936,13 @@
         <v>506</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>457</v>
+        <v>328</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>455</v>
+        <v>322</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>456</v>
+        <v>16</v>
       </c>
       <c r="G129" s="3" t="s">
         <v>17</v>
@@ -8945,13 +8960,13 @@
         <v>506</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>419</v>
+        <v>328</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>348</v>
+        <v>323</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="G130" s="3" t="s">
         <v>17</v>
@@ -8969,13 +8984,13 @@
         <v>506</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>419</v>
+        <v>328</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>349</v>
+        <v>324</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>350</v>
+        <v>17</v>
       </c>
       <c r="G131" s="3" t="s">
         <v>17</v>
@@ -8993,13 +9008,13 @@
         <v>506</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>348</v>
+        <v>268</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>18</v>
+        <v>329</v>
       </c>
       <c r="G132" s="3" t="s">
         <v>17</v>
@@ -9017,13 +9032,13 @@
         <v>506</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>349</v>
+        <v>269</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>350</v>
+        <v>329</v>
       </c>
       <c r="G133" s="3" t="s">
         <v>17</v>
@@ -9041,13 +9056,13 @@
         <v>506</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>351</v>
+        <v>454</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>348</v>
+        <v>455</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>17</v>
+        <v>456</v>
       </c>
       <c r="G134" s="3" t="s">
         <v>17</v>
@@ -9065,13 +9080,13 @@
         <v>506</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>351</v>
+        <v>457</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>349</v>
+        <v>455</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>350</v>
+        <v>456</v>
       </c>
       <c r="G135" s="3" t="s">
         <v>17</v>
@@ -9089,13 +9104,13 @@
         <v>506</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>502</v>
+        <v>419</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F136" s="3">
-        <v>20</v>
+        <v>348</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="G136" s="3" t="s">
         <v>17</v>
@@ -9113,13 +9128,13 @@
         <v>506</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>503</v>
+        <v>419</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F137" s="3">
-        <v>200</v>
+        <v>349</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>350</v>
       </c>
       <c r="G137" s="3" t="s">
         <v>17</v>
@@ -9137,13 +9152,13 @@
         <v>506</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>221</v>
+        <v>347</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>228</v>
+        <v>348</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G138" s="3" t="s">
         <v>17</v>
@@ -9161,13 +9176,13 @@
         <v>506</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>221</v>
+        <v>347</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>229</v>
+        <v>349</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>57</v>
+        <v>350</v>
       </c>
       <c r="G139" s="3" t="s">
         <v>17</v>
@@ -9185,12 +9200,14 @@
         <v>506</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>221</v>
+        <v>351</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="F140" s="3"/>
+        <v>348</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="G140" s="3" t="s">
         <v>17</v>
       </c>
@@ -9207,13 +9224,13 @@
         <v>506</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>221</v>
+        <v>351</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>230</v>
+        <v>349</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>39</v>
+        <v>350</v>
       </c>
       <c r="G141" s="3" t="s">
         <v>17</v>
@@ -9231,13 +9248,13 @@
         <v>506</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>221</v>
+        <v>502</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="F142" s="3" t="s">
-        <v>39</v>
+        <v>107</v>
+      </c>
+      <c r="F142" s="3">
+        <v>20</v>
       </c>
       <c r="G142" s="3" t="s">
         <v>17</v>
@@ -9255,13 +9272,13 @@
         <v>506</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>221</v>
+        <v>503</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="F143" s="3" t="s">
-        <v>250</v>
+        <v>107</v>
+      </c>
+      <c r="F143" s="3">
+        <v>200</v>
       </c>
       <c r="G143" s="3" t="s">
         <v>17</v>
@@ -9282,10 +9299,10 @@
         <v>221</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>251</v>
+        <v>17</v>
       </c>
       <c r="G144" s="3" t="s">
         <v>17</v>
@@ -9306,10 +9323,10 @@
         <v>221</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>252</v>
+        <v>57</v>
       </c>
       <c r="G145" s="3" t="s">
         <v>17</v>
@@ -9327,14 +9344,12 @@
         <v>506</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>169</v>
+        <v>221</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="F146" s="3" t="s">
-        <v>178</v>
-      </c>
+        <v>278</v>
+      </c>
+      <c r="F146" s="3"/>
       <c r="G146" s="3" t="s">
         <v>17</v>
       </c>
@@ -9351,13 +9366,13 @@
         <v>506</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>169</v>
+        <v>221</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>171</v>
+        <v>230</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>394</v>
+        <v>39</v>
       </c>
       <c r="G147" s="3" t="s">
         <v>17</v>
@@ -9375,13 +9390,13 @@
         <v>506</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>169</v>
+        <v>221</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>172</v>
+        <v>231</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="G148" s="3" t="s">
         <v>17</v>
@@ -9399,13 +9414,13 @@
         <v>506</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>169</v>
+        <v>221</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>173</v>
+        <v>249</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>38</v>
+        <v>250</v>
       </c>
       <c r="G149" s="3" t="s">
         <v>17</v>
@@ -9423,13 +9438,13 @@
         <v>506</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>174</v>
+        <v>221</v>
       </c>
       <c r="E150" s="3" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>168</v>
+        <v>251</v>
       </c>
       <c r="G150" s="3" t="s">
         <v>17</v>
@@ -9447,13 +9462,13 @@
         <v>506</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>174</v>
+        <v>221</v>
       </c>
       <c r="E151" s="3" t="s">
-        <v>177</v>
+        <v>227</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>168</v>
+        <v>252</v>
       </c>
       <c r="G151" s="3" t="s">
         <v>17</v>
@@ -9471,13 +9486,13 @@
         <v>506</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E152" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G152" s="3" t="s">
         <v>17</v>
@@ -9495,13 +9510,13 @@
         <v>506</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E153" s="3" t="s">
-        <v>274</v>
+        <v>171</v>
       </c>
       <c r="F153" s="3" t="s">
-        <v>179</v>
+        <v>394</v>
       </c>
       <c r="G153" s="3" t="s">
         <v>17</v>
@@ -9519,13 +9534,13 @@
         <v>506</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="E154" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F154" s="3">
-        <v>1500</v>
+        <v>172</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="G154" s="3" t="s">
         <v>17</v>
@@ -9543,13 +9558,13 @@
         <v>506</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="E155" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="F155" s="3">
-        <v>600</v>
+        <v>173</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="G155" s="3" t="s">
         <v>17</v>
@@ -9567,13 +9582,13 @@
         <v>506</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>129</v>
+        <v>174</v>
       </c>
       <c r="E156" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="F156" s="3">
-        <v>2000</v>
+        <v>175</v>
+      </c>
+      <c r="F156" s="3" t="s">
+        <v>168</v>
       </c>
       <c r="G156" s="3" t="s">
         <v>17</v>
@@ -9591,13 +9606,13 @@
         <v>506</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>129</v>
+        <v>174</v>
       </c>
       <c r="E157" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="F157" s="3">
-        <v>3000</v>
+        <v>177</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>168</v>
       </c>
       <c r="G157" s="3" t="s">
         <v>17</v>
@@ -9615,13 +9630,13 @@
         <v>506</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>129</v>
+        <v>174</v>
       </c>
       <c r="E158" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="F158" s="3">
-        <v>400</v>
+        <v>176</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>179</v>
       </c>
       <c r="G158" s="3" t="s">
         <v>17</v>
@@ -9639,13 +9654,13 @@
         <v>506</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="E159" s="3" t="s">
-        <v>181</v>
+        <v>274</v>
       </c>
       <c r="F159" s="3" t="s">
-        <v>17</v>
+        <v>179</v>
       </c>
       <c r="G159" s="3" t="s">
         <v>17</v>
@@ -9663,13 +9678,13 @@
         <v>506</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>184</v>
+        <v>129</v>
       </c>
       <c r="E160" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="F160" s="3" t="s">
-        <v>385</v>
+        <v>130</v>
+      </c>
+      <c r="F160" s="3">
+        <v>1500</v>
       </c>
       <c r="G160" s="3" t="s">
         <v>17</v>
@@ -9687,13 +9702,13 @@
         <v>506</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>356</v>
+        <v>129</v>
       </c>
       <c r="E161" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="F161" s="3" t="s">
-        <v>255</v>
+        <v>131</v>
+      </c>
+      <c r="F161" s="3">
+        <v>600</v>
       </c>
       <c r="G161" s="3" t="s">
         <v>17</v>
@@ -9711,13 +9726,13 @@
         <v>506</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>356</v>
+        <v>129</v>
       </c>
       <c r="E162" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="F162" s="3" t="s">
-        <v>363</v>
+        <v>132</v>
+      </c>
+      <c r="F162" s="3">
+        <v>2000</v>
       </c>
       <c r="G162" s="3" t="s">
         <v>17</v>
@@ -9735,13 +9750,13 @@
         <v>506</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>356</v>
+        <v>129</v>
       </c>
       <c r="E163" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="F163" s="3" t="s">
-        <v>362</v>
+        <v>133</v>
+      </c>
+      <c r="F163" s="3">
+        <v>3000</v>
       </c>
       <c r="G163" s="3" t="s">
         <v>17</v>
@@ -9759,13 +9774,13 @@
         <v>506</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>356</v>
+        <v>129</v>
       </c>
       <c r="E164" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="F164" s="3" t="s">
-        <v>361</v>
+        <v>134</v>
+      </c>
+      <c r="F164" s="3">
+        <v>400</v>
       </c>
       <c r="G164" s="3" t="s">
         <v>17</v>
@@ -9783,13 +9798,13 @@
         <v>506</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>356</v>
+        <v>180</v>
       </c>
       <c r="E165" s="3" t="s">
-        <v>359</v>
+        <v>181</v>
       </c>
       <c r="F165" s="3" t="s">
-        <v>360</v>
+        <v>17</v>
       </c>
       <c r="G165" s="3" t="s">
         <v>17</v>
@@ -9807,13 +9822,13 @@
         <v>506</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="E166" s="3" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="F166" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="G166" s="3" t="s">
         <v>17</v>
@@ -9831,13 +9846,13 @@
         <v>506</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>199</v>
+        <v>356</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>197</v>
+        <v>268</v>
       </c>
       <c r="F167" s="3" t="s">
-        <v>217</v>
+        <v>255</v>
       </c>
       <c r="G167" s="3" t="s">
         <v>17</v>
@@ -9855,13 +9870,13 @@
         <v>506</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>199</v>
+        <v>356</v>
       </c>
       <c r="E168" s="3" t="s">
-        <v>196</v>
+        <v>269</v>
       </c>
       <c r="F168" s="3" t="s">
-        <v>17</v>
+        <v>363</v>
       </c>
       <c r="G168" s="3" t="s">
         <v>17</v>
@@ -9879,13 +9894,13 @@
         <v>506</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>200</v>
+        <v>356</v>
       </c>
       <c r="E169" s="3" t="s">
-        <v>195</v>
+        <v>357</v>
       </c>
       <c r="F169" s="3" t="s">
-        <v>386</v>
+        <v>362</v>
       </c>
       <c r="G169" s="3" t="s">
         <v>17</v>
@@ -9903,13 +9918,13 @@
         <v>506</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>200</v>
+        <v>356</v>
       </c>
       <c r="E170" s="3" t="s">
-        <v>197</v>
+        <v>358</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>217</v>
+        <v>361</v>
       </c>
       <c r="G170" s="3" t="s">
         <v>17</v>
@@ -9927,13 +9942,13 @@
         <v>506</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>200</v>
+        <v>356</v>
       </c>
       <c r="E171" s="3" t="s">
-        <v>196</v>
+        <v>359</v>
       </c>
       <c r="F171" s="3" t="s">
-        <v>17</v>
+        <v>360</v>
       </c>
       <c r="G171" s="3" t="s">
         <v>17</v>
@@ -9951,7 +9966,7 @@
         <v>506</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E172" s="3" t="s">
         <v>195</v>
@@ -9975,13 +9990,13 @@
         <v>506</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E173" s="3" t="s">
         <v>196</v>
       </c>
       <c r="F173" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G173" s="3" t="s">
         <v>17</v>
@@ -9999,13 +10014,13 @@
         <v>506</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="E174" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>217</v>
+        <v>386</v>
       </c>
       <c r="G174" s="3" t="s">
         <v>17</v>
@@ -10023,13 +10038,13 @@
         <v>506</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F175" s="3" t="s">
-        <v>386</v>
+        <v>17</v>
       </c>
       <c r="G175" s="3" t="s">
         <v>17</v>
@@ -10047,13 +10062,13 @@
         <v>506</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E176" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>18</v>
+        <v>387</v>
       </c>
       <c r="G176" s="3" t="s">
         <v>17</v>
@@ -10071,13 +10086,13 @@
         <v>506</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E177" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F177" s="3" t="s">
-        <v>217</v>
+        <v>18</v>
       </c>
       <c r="G177" s="3" t="s">
         <v>17</v>
@@ -10095,13 +10110,13 @@
         <v>506</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E178" s="3" t="s">
         <v>195</v>
       </c>
       <c r="F178" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G178" s="3" t="s">
         <v>17</v>
@@ -10119,7 +10134,7 @@
         <v>506</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E179" s="3" t="s">
         <v>196</v>
@@ -10146,10 +10161,10 @@
         <v>201</v>
       </c>
       <c r="E180" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F180" s="3" t="s">
-        <v>217</v>
+        <v>387</v>
       </c>
       <c r="G180" s="3" t="s">
         <v>17</v>
@@ -10167,13 +10182,13 @@
         <v>506</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E181" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F181" s="3" t="s">
-        <v>386</v>
+        <v>18</v>
       </c>
       <c r="G181" s="3" t="s">
         <v>17</v>
@@ -10194,10 +10209,10 @@
         <v>202</v>
       </c>
       <c r="E182" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F182" s="3" t="s">
-        <v>18</v>
+        <v>386</v>
       </c>
       <c r="G182" s="3" t="s">
         <v>17</v>
@@ -10218,10 +10233,10 @@
         <v>202</v>
       </c>
       <c r="E183" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F183" s="3" t="s">
-        <v>217</v>
+        <v>18</v>
       </c>
       <c r="G183" s="3" t="s">
         <v>17</v>
@@ -12923,13 +12938,13 @@
         <v>505</v>
       </c>
       <c r="D296" s="9" t="s">
-        <v>507</v>
+        <v>537</v>
       </c>
       <c r="E296" s="9" t="s">
-        <v>508</v>
+        <v>536</v>
       </c>
       <c r="F296" s="9" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G296" s="9" t="s">
         <v>17</v>
@@ -12950,10 +12965,10 @@
         <v>507</v>
       </c>
       <c r="E297" s="9" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F297" s="9" t="s">
-        <v>535</v>
+        <v>18</v>
       </c>
       <c r="G297" s="9" t="s">
         <v>17</v>
@@ -12974,10 +12989,10 @@
         <v>507</v>
       </c>
       <c r="E298" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F298" s="9" t="s">
-        <v>511</v>
+        <v>535</v>
       </c>
       <c r="G298" s="9" t="s">
         <v>17</v>
@@ -12995,13 +13010,13 @@
         <v>505</v>
       </c>
       <c r="D299" s="9" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
       <c r="E299" s="9" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="F299" s="9" t="s">
-        <v>18</v>
+        <v>511</v>
       </c>
       <c r="G299" s="9" t="s">
         <v>17</v>
@@ -13022,10 +13037,10 @@
         <v>513</v>
       </c>
       <c r="E300" s="9" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F300" s="9" t="s">
-        <v>535</v>
+        <v>18</v>
       </c>
       <c r="G300" s="9" t="s">
         <v>17</v>
@@ -13046,10 +13061,10 @@
         <v>513</v>
       </c>
       <c r="E301" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F301" s="9" t="s">
-        <v>511</v>
+        <v>535</v>
       </c>
       <c r="G301" s="9" t="s">
         <v>17</v>
@@ -13067,13 +13082,13 @@
         <v>505</v>
       </c>
       <c r="D302" s="9" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E302" s="9" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="F302" s="9" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="G302" s="9" t="s">
         <v>17</v>
@@ -13094,7 +13109,7 @@
         <v>512</v>
       </c>
       <c r="E303" s="9" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>515</v>
@@ -13118,10 +13133,10 @@
         <v>512</v>
       </c>
       <c r="E304" s="9" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F304" s="9" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="G304" s="9" t="s">
         <v>17</v>
@@ -13142,10 +13157,10 @@
         <v>512</v>
       </c>
       <c r="E305" s="9" t="s">
-        <v>279</v>
+        <v>517</v>
       </c>
       <c r="F305" s="9" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="G305" s="9" t="s">
         <v>17</v>
@@ -13166,10 +13181,10 @@
         <v>512</v>
       </c>
       <c r="E306" s="9" t="s">
-        <v>520</v>
+        <v>279</v>
       </c>
       <c r="F306" s="9" t="s">
-        <v>17</v>
+        <v>519</v>
       </c>
       <c r="G306" s="9" t="s">
         <v>17</v>
@@ -13190,7 +13205,7 @@
         <v>512</v>
       </c>
       <c r="E307" s="9" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>17</v>
@@ -13211,13 +13226,13 @@
         <v>505</v>
       </c>
       <c r="D308" s="9" t="s">
-        <v>522</v>
+        <v>512</v>
       </c>
       <c r="E308" s="9" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="F308" s="9" t="s">
-        <v>524</v>
+        <v>17</v>
       </c>
       <c r="G308" s="9" t="s">
         <v>17</v>
@@ -13238,10 +13253,10 @@
         <v>522</v>
       </c>
       <c r="E309" s="9" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="F309" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="G309" s="9" t="s">
         <v>17</v>
@@ -13262,10 +13277,10 @@
         <v>522</v>
       </c>
       <c r="E310" s="9" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="F310" s="9" t="s">
-        <v>37</v>
+        <v>526</v>
       </c>
       <c r="G310" s="9" t="s">
         <v>17</v>
@@ -13286,10 +13301,10 @@
         <v>522</v>
       </c>
       <c r="E311" s="9" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F311" s="9" t="s">
-        <v>529</v>
+        <v>37</v>
       </c>
       <c r="G311" s="9" t="s">
         <v>17</v>
@@ -13307,13 +13322,13 @@
         <v>505</v>
       </c>
       <c r="D312" s="9" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="E312" s="9" t="s">
-        <v>42</v>
+        <v>528</v>
       </c>
       <c r="F312" s="9" t="s">
-        <v>17</v>
+        <v>529</v>
       </c>
       <c r="G312" s="9" t="s">
         <v>17</v>
@@ -13334,10 +13349,10 @@
         <v>530</v>
       </c>
       <c r="E313" s="9" t="s">
-        <v>531</v>
+        <v>42</v>
       </c>
       <c r="F313" s="9" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="G313" s="9" t="s">
         <v>17</v>
@@ -13358,7 +13373,7 @@
         <v>530</v>
       </c>
       <c r="E314" s="9" t="s">
-        <v>52</v>
+        <v>531</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>72</v>
@@ -13382,10 +13397,10 @@
         <v>530</v>
       </c>
       <c r="E315" s="9" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="F315" s="9" t="s">
-        <v>305</v>
+        <v>72</v>
       </c>
       <c r="G315" s="9" t="s">
         <v>17</v>
@@ -13406,10 +13421,10 @@
         <v>530</v>
       </c>
       <c r="E316" s="9" t="s">
-        <v>532</v>
+        <v>66</v>
       </c>
       <c r="F316" s="9" t="s">
-        <v>39</v>
+        <v>305</v>
       </c>
       <c r="G316" s="9" t="s">
         <v>17</v>
@@ -13430,18 +13445,42 @@
         <v>530</v>
       </c>
       <c r="E317" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="F317" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G317" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H317" s="9"/>
+    </row>
+    <row r="318" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A318" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="B318" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="C318" s="9" t="s">
+        <v>505</v>
+      </c>
+      <c r="D318" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="E318" s="9" t="s">
         <v>533</v>
       </c>
-      <c r="F317" s="9" t="s">
+      <c r="F318" s="9" t="s">
         <v>534</v>
       </c>
-      <c r="G317" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H317" s="9"/>
+      <c r="G318" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H318" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G286" xr:uid="{04129BFA-1C57-4A9F-9E8B-6ECAA0BFBBBF}"/>
+  <autoFilter ref="A1:G318" xr:uid="{04129BFA-1C57-4A9F-9E8B-6ECAA0BFBBBF}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>